<commit_message>
add new table employee and match platform
</commit_message>
<xml_diff>
--- a/Project-QM/QBOS_W12.xlsx
+++ b/Project-QM/QBOS_W12.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtinoco2\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francisco\Downloads\Failures-PMI\Project-QM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278A82FE-89E2-4020-A14D-3540C5AA7C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41804BA8-98FA-4B0E-8607-083DD9300699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="34">
   <si>
     <t>Personnel Name</t>
   </si>
@@ -122,12 +122,6 @@
   </si>
   <si>
     <t>Victor Zuniga</t>
-  </si>
-  <si>
-    <t>Applied filters:
-AUTHOR is not (Blank)
-Department  is Filtros Capsula
-DATE LOCAL is on or after 3/16/2026 and is before 3/20/2026</t>
   </si>
 </sst>
 </file>
@@ -191,7 +185,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -507,8 +501,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E30"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -924,11 +918,6 @@
       </c>
       <c r="E28" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>